<commit_message>
fix: resolve Unit Head redirection error and cleanup document IDs
</commit_message>
<xml_diff>
--- a/Code Tables/Database_Formats.xlsx
+++ b/Code Tables/Database_Formats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shalomjadee.dikit/Documents/pds_dashboard_task/Code Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D5A1E9-632D-1F44-B1A0-3AE09495E271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B64B11C-7D85-4644-93D9-0AFF4C41200C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5540" yWindow="2300" windowWidth="27700" windowHeight="16940" activeTab="1" xr2:uid="{D532F848-C0D2-E748-9988-BC9DDAEF8A71}"/>
+    <workbookView xWindow="5540" yWindow="2300" windowWidth="27700" windowHeight="16940" xr2:uid="{D532F848-C0D2-E748-9988-BC9DDAEF8A71}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="1" r:id="rId1"/>

</xml_diff>